<commit_message>
[new] attack pipline base
</commit_message>
<xml_diff>
--- a/table_config/_tables/__enums__.xlsx
+++ b/table_config/_tables/__enums__.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
   <si>
     <t>##var</t>
   </si>
@@ -104,6 +104,24 @@
     <t>攻击</t>
   </si>
   <si>
+    <t>Defence</t>
+  </si>
+  <si>
+    <t>防御</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>精准</t>
+  </si>
+  <si>
+    <t>Dexterity</t>
+  </si>
+  <si>
+    <t>敏捷</t>
+  </si>
+  <si>
     <t>Battle.Tag</t>
   </si>
   <si>
@@ -111,6 +129,12 @@
   </si>
   <si>
     <t>免疫所有伤害</t>
+  </si>
+  <si>
+    <t>Dead</t>
+  </si>
+  <si>
+    <t>死亡</t>
   </si>
   <si>
     <t>Battle.DamageSource</t>
@@ -1133,7 +1157,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="6.45833333333333" customWidth="1"/>
@@ -1294,36 +1318,41 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="5"/>
+      <c r="H6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="6">
+        <v>3</v>
+      </c>
+      <c r="K6" s="5" t="str">
+        <f>I6</f>
+        <v>防御</v>
+      </c>
       <c r="L6" s="5"/>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J7" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K7" s="5" t="str">
         <f>I7</f>
-        <v>免疫所有伤害</v>
+        <v>精准</v>
       </c>
       <c r="L7" s="5"/>
     </row>
@@ -1335,61 +1364,64 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" s="6">
+        <v>5</v>
+      </c>
+      <c r="K8" s="5" t="str">
+        <f>I8</f>
+        <v>敏捷</v>
+      </c>
       <c r="L8" s="5"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="B9" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
-      <c r="E9" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" s="6">
-        <v>1</v>
-      </c>
-      <c r="K9" s="5" t="str">
-        <f>I9</f>
-        <v>主要伤害</v>
-      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="5"/>
       <c r="L9" s="5"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="B10" s="5"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J10" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="5" t="str">
         <f>I10</f>
-        <v>派生伤害</v>
+        <v>免疫所有伤害</v>
       </c>
       <c r="L10" s="5"/>
     </row>
     <row r="11" spans="1:12">
+      <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -1397,21 +1429,22 @@
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J11" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" s="5" t="str">
         <f>I11</f>
-        <v>反弹伤害</v>
+        <v>死亡</v>
       </c>
       <c r="L11" s="5"/>
     </row>
     <row r="12" spans="1:12">
+      <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -1426,7 +1459,7 @@
     </row>
     <row r="13" spans="1:12">
       <c r="B13" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -1436,17 +1469,17 @@
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
       <c r="H13" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J13" s="6">
         <v>1</v>
       </c>
       <c r="K13" s="5" t="str">
         <f>I13</f>
-        <v>物理伤害</v>
+        <v>主要伤害</v>
       </c>
       <c r="L13" s="5"/>
     </row>
@@ -1458,17 +1491,17 @@
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J14" s="6">
         <v>2</v>
       </c>
       <c r="K14" s="5" t="str">
         <f>I14</f>
-        <v>魔法伤害</v>
+        <v>派生伤害</v>
       </c>
       <c r="L14" s="5"/>
     </row>
@@ -1479,49 +1512,58 @@
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="5"/>
+      <c r="H15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J15" s="6">
+        <v>3</v>
+      </c>
+      <c r="K15" s="5" t="str">
+        <f>I15</f>
+        <v>反弹伤害</v>
+      </c>
       <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:12">
-      <c r="B16" s="5" t="s">
-        <v>40</v>
-      </c>
+      <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="J16" s="6">
-        <v>1</v>
-      </c>
-      <c r="K16" s="5" t="str">
-        <f>I16</f>
-        <v>基础毒伤害</v>
-      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="5"/>
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:12">
-      <c r="B17" s="5"/>
+      <c r="B17" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="E17" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="5"/>
+      <c r="H17" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J17" s="6">
+        <v>1</v>
+      </c>
+      <c r="K17" s="5" t="str">
+        <f>I17</f>
+        <v>物理伤害</v>
+      </c>
       <c r="L17" s="5"/>
     </row>
     <row r="18" spans="1:12">
@@ -1531,10 +1573,19 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="5"/>
+      <c r="H18" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="J18" s="6">
+        <v>2</v>
+      </c>
+      <c r="K18" s="5" t="str">
+        <f>I18</f>
+        <v>魔法伤害</v>
+      </c>
       <c r="L18" s="5"/>
     </row>
     <row r="19" spans="1:12">
@@ -1551,16 +1602,29 @@
       <c r="L19" s="5"/>
     </row>
     <row r="20" spans="1:12">
-      <c r="B20" s="5"/>
+      <c r="B20" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="E20" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
+      <c r="H20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J20" s="6">
+        <v>1</v>
+      </c>
+      <c r="K20" s="5" t="str">
+        <f>I20</f>
+        <v>基础毒伤害</v>
+      </c>
       <c r="L20" s="5"/>
     </row>
     <row r="21" spans="1:12">
@@ -1612,7 +1676,7 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="6"/>
-      <c r="K24" s="5"/>
+      <c r="K24" s="6"/>
       <c r="L24" s="5"/>
     </row>
     <row r="25" spans="1:12">
@@ -1642,7 +1706,6 @@
       <c r="L26" s="5"/>
     </row>
     <row r="27" spans="1:12">
-      <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -1656,7 +1719,6 @@
       <c r="L27" s="5"/>
     </row>
     <row r="28" spans="1:12">
-      <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
@@ -1696,6 +1758,7 @@
       <c r="L30" s="5"/>
     </row>
     <row r="31" spans="1:12">
+      <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -1709,6 +1772,7 @@
       <c r="L31" s="5"/>
     </row>
     <row r="32" spans="1:12">
+      <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -2527,6 +2591,58 @@
       <c r="K94" s="5"/>
       <c r="L94" s="5"/>
     </row>
+    <row r="95" spans="2:12">
+      <c r="B95" s="5"/>
+      <c r="C95" s="5"/>
+      <c r="D95" s="5"/>
+      <c r="E95" s="5"/>
+      <c r="F95" s="5"/>
+      <c r="G95" s="5"/>
+      <c r="H95" s="5"/>
+      <c r="I95" s="5"/>
+      <c r="J95" s="6"/>
+      <c r="K95" s="5"/>
+      <c r="L95" s="5"/>
+    </row>
+    <row r="96" spans="2:12">
+      <c r="B96" s="5"/>
+      <c r="C96" s="5"/>
+      <c r="D96" s="5"/>
+      <c r="E96" s="5"/>
+      <c r="F96" s="5"/>
+      <c r="G96" s="5"/>
+      <c r="H96" s="5"/>
+      <c r="I96" s="5"/>
+      <c r="J96" s="6"/>
+      <c r="K96" s="5"/>
+      <c r="L96" s="5"/>
+    </row>
+    <row r="97" spans="2:12">
+      <c r="B97" s="5"/>
+      <c r="C97" s="5"/>
+      <c r="D97" s="5"/>
+      <c r="E97" s="5"/>
+      <c r="F97" s="5"/>
+      <c r="G97" s="5"/>
+      <c r="H97" s="5"/>
+      <c r="I97" s="5"/>
+      <c r="J97" s="6"/>
+      <c r="K97" s="5"/>
+      <c r="L97" s="5"/>
+    </row>
+    <row r="98" spans="2:12">
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5"/>
+      <c r="E98" s="5"/>
+      <c r="F98" s="5"/>
+      <c r="G98" s="5"/>
+      <c r="H98" s="5"/>
+      <c r="I98" s="5"/>
+      <c r="J98" s="6"/>
+      <c r="K98" s="5"/>
+      <c r="L98" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="H1:L1"/>

</xml_diff>